<commit_message>
Enhance job selector with tracking sheet fields and per-job edits.
Parse Paper GSM columns, fix multi-field search, add per-job remarks and no of cuts, and match marketing site header branding.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/sample-jobs.xlsx
+++ b/public/sample-jobs.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Jobs" sheetId="1" r:id="rId1"/>
+    <sheet name="Boxes" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:M3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,105 +407,124 @@
         <v>Box Name</v>
       </c>
       <c r="C1" t="str">
-        <v>Box ID</v>
+        <v>Number of Layers (1,3,5,7)</v>
       </c>
       <c r="D1" t="str">
-        <v>Dimensions</v>
+        <v>Dimensions (L X W X H) in MM</v>
       </c>
       <c r="E1" t="str">
-        <v>Layers</v>
+        <v>Reel size (Inch) Width X Diameter</v>
       </c>
       <c r="F1" t="str">
-        <v>Reel Size</v>
+        <v>CUT SIZE MM</v>
       </c>
       <c r="G1" t="str">
-        <v>Remarks/Notes</v>
+        <v>Paper BF</v>
       </c>
       <c r="H1" t="str">
-        <v>Proceed to Manufacture</v>
+        <v>Face</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Flute</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Kraft</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Flute</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Kraft</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Color Job (1/2/3/4/6)</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ABC Industries</v>
+        <v>Rakesh ji</v>
       </c>
       <c r="B2" t="str">
-        <v>Corrugated Box A</v>
+        <v>Raw Sheets</v>
       </c>
       <c r="C2" t="str">
-        <v>BOX-001</v>
+        <v>3 Ply</v>
       </c>
       <c r="D2" t="str">
-        <v>12x10x8</v>
+        <v>1042x306x645</v>
       </c>
       <c r="E2" t="str">
-        <v>3</v>
+        <v>38.2</v>
       </c>
       <c r="F2" t="str">
-        <v>1200</v>
+        <v>1380</v>
       </c>
       <c r="G2" t="str">
-        <v>Handle with care</v>
+        <v>18</v>
       </c>
       <c r="H2" t="str">
-        <v>Yes</v>
+        <v>180</v>
+      </c>
+      <c r="I2" t="str">
+        <v>140</v>
+      </c>
+      <c r="J2" t="str">
+        <v>140</v>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v>N/A</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>XYZ Traders</v>
+        <v>Metro money</v>
       </c>
       <c r="B3" t="str">
-        <v>Export Box B</v>
+        <v>6 X 9</v>
       </c>
       <c r="C3" t="str">
-        <v>BOX-002</v>
+        <v>5 Ply</v>
       </c>
       <c r="D3" t="str">
-        <v>18x14x12</v>
+        <v>786 x 458 x 508</v>
       </c>
       <c r="E3" t="str">
-        <v>5</v>
+        <v>41.4</v>
       </c>
       <c r="F3" t="str">
-        <v>1500</v>
+        <v>2595</v>
       </c>
       <c r="G3" t="str">
-        <v>Urgent order</v>
+        <v>22</v>
       </c>
       <c r="H3" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Prime Foods</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Food Grade Box</v>
-      </c>
-      <c r="C4" t="str">
-        <v>BOX-003</v>
-      </c>
-      <c r="D4" t="str">
-        <v>10x8x6</v>
-      </c>
-      <c r="E4" t="str">
-        <v>2</v>
-      </c>
-      <c r="F4" t="str">
-        <v>900</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Food safe laminate</v>
-      </c>
-      <c r="H4" t="str">
-        <v>No</v>
+        <v>140</v>
+      </c>
+      <c r="I3" t="str">
+        <v>120</v>
+      </c>
+      <c r="J3" t="str">
+        <v>120</v>
+      </c>
+      <c r="K3" t="str">
+        <v>120</v>
+      </c>
+      <c r="L3" t="str">
+        <v>120</v>
+      </c>
+      <c r="M3" t="str">
+        <v>YES</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>